<commit_message>
Update as-build drawing v1.06
Увеличил число позиции
</commit_message>
<xml_diff>
--- a/ВОР.xlsx
+++ b/ВОР.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="38">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -108,9 +108,6 @@
     <t>Объем, м²</t>
   </si>
   <si>
-    <t>Шпаклевка финишная</t>
-  </si>
-  <si>
     <t xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </t>
   </si>
   <si>
@@ -127,6 +124,12 @@
   </si>
   <si>
     <t>Монтаж углового профиля</t>
+  </si>
+  <si>
+    <t>Шпаклевка финишная по ГВЛ</t>
+  </si>
+  <si>
+    <t>Шпаклевка финишная по оштукатуренной поверхности</t>
   </si>
 </sst>
 </file>
@@ -311,9 +314,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -337,6 +337,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -792,7 +795,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A4:E69"/>
+  <dimension ref="A4:E75"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="9" customWidth="1"/>
@@ -942,11 +945,12 @@
         <v>3</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D19" s="17">
         <v>178.11</v>
       </c>
+      <c r="E19" s="34"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B20" s="15">
@@ -955,468 +959,536 @@
       <c r="C20" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>28</v>
-      </c>
+      <c r="D20" s="17">
+        <v>0</v>
+      </c>
+      <c r="E20" s="34"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B21" s="15">
         <v>5</v>
       </c>
-      <c r="C21" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="17">
+      <c r="C21" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B22" s="15">
+        <v>6</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="17">
         <f>D17</f>
         <v>178.11</v>
       </c>
-      <c r="E21" s="13">
-        <v>9003</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="9" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B24" s="10"/>
-      <c r="C24" s="11" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="10"/>
+      <c r="C25" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="12"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B25" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="16" t="s">
+      <c r="D25" s="12"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B26" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D26" s="17" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B26" s="15">
-        <v>1</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="17">
-        <v>340.88</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B27" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D27" s="17">
-        <v>0</v>
+        <v>340.88</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B28" s="15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D28" s="17">
-        <f>D26</f>
-        <v>340.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B29" s="15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="17" t="s">
-        <v>27</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="D29" s="17">
+        <v>340.88</v>
+      </c>
+      <c r="E29" s="34"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B30" s="15">
+        <v>4</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="17">
+        <v>0</v>
+      </c>
+      <c r="E30" s="34"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B31" s="15">
         <v>5</v>
       </c>
-      <c r="C30" s="23" t="str">
-        <f>C21</f>
+      <c r="C31" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="15">
+        <v>6</v>
+      </c>
+      <c r="C32" s="23" t="str">
+        <f>C22</f>
         <v xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </v>
       </c>
-      <c r="D30" s="17">
-        <f>D26</f>
+      <c r="D32" s="17">
+        <f>D27</f>
         <v>340.88</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="9" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B33" s="10"/>
-      <c r="C33" s="11" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="10"/>
+      <c r="C35" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D33" s="12"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B34" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="16" t="s">
+      <c r="D35" s="12"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D34" s="17" t="s">
+      <c r="D36" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B35" s="15">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B37" s="15">
         <v>1</v>
       </c>
-      <c r="C35" s="16" t="s">
+      <c r="C37" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="17">
+      <c r="D37" s="17">
         <v>192.99</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B36" s="15">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B38" s="15">
         <v>2</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C38" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D36" s="17">
+      <c r="D38" s="17">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B37" s="15">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B39" s="15">
         <v>3</v>
       </c>
-      <c r="C37" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D37" s="17">
-        <f>D35</f>
+      <c r="C39" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="17">
         <v>192.99</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B38" s="15">
+      <c r="E39" s="34"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="15">
         <v>4</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C40" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D40" s="17">
+        <v>0</v>
+      </c>
+      <c r="E40" s="34"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B41" s="15">
+        <v>5</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B39" s="15">
-        <v>5</v>
-      </c>
-      <c r="C39" s="23" t="str">
-        <f>C30</f>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B42" s="15">
+        <v>6</v>
+      </c>
+      <c r="C42" s="23" t="str">
+        <f>C32</f>
         <v xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </v>
       </c>
-      <c r="D39" s="17">
-        <f>D35</f>
+      <c r="D42" s="17">
+        <f>D37</f>
         <v>192.99</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B40" s="19"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="21"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="9" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B43" s="19"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="21"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B43" s="10"/>
-      <c r="C43" s="11" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B46" s="10"/>
+      <c r="C46" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D43" s="12"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B44" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="16" t="s">
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B47" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="17" t="s">
+      <c r="D47" s="17" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B45" s="15">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B48" s="15">
         <v>1</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C48" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="17">
+      <c r="D48" s="17">
         <v>246.3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B46" s="15">
-        <v>2</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D46" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B47" s="15">
-        <v>3</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D47" s="17">
-        <f>D45</f>
-        <v>246.3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B48" s="15">
-        <v>4</v>
-      </c>
-      <c r="C48" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B49" s="15">
+        <v>2</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="15">
+        <v>3</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D50" s="17">
+        <v>246.3</v>
+      </c>
+      <c r="E50" s="34"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B51" s="15">
+        <v>4</v>
+      </c>
+      <c r="C51" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D51" s="17">
+        <v>0</v>
+      </c>
+      <c r="E51" s="34"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B52" s="15">
         <v>5</v>
       </c>
-      <c r="C49" s="23" t="str">
-        <f>C39</f>
+      <c r="C52" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B53" s="15">
+        <v>6</v>
+      </c>
+      <c r="C53" s="23" t="str">
+        <f>C42</f>
         <v xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </v>
       </c>
-      <c r="D49" s="17">
-        <f>D45</f>
+      <c r="D53" s="17">
+        <f>D48</f>
         <v>246.3</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="9" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B52" s="10"/>
-      <c r="C52" s="11" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B56" s="10"/>
+      <c r="C56" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D52" s="12"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B53" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C53" s="16" t="s">
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B57" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D53" s="17" t="s">
+      <c r="D57" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B54" s="15">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B58" s="15">
         <v>1</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C58" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D54" s="17">
+      <c r="D58" s="17">
         <v>105.63</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B55" s="15">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B59" s="15">
         <v>2</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C59" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="17">
+      <c r="D59" s="17">
         <v>4.1500000000000004</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="15">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B60" s="15">
         <v>3</v>
       </c>
-      <c r="C56" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D56" s="17">
-        <f>D54+D55</f>
+      <c r="C60" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D60" s="17">
+        <v>105.63</v>
+      </c>
+      <c r="E60" s="34"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B61" s="15">
+        <v>4</v>
+      </c>
+      <c r="C61" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D61" s="17">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="E61" s="34"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B62" s="15">
+        <v>5</v>
+      </c>
+      <c r="C62" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D62" s="17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="25"/>
+      <c r="B63" s="15">
+        <v>6</v>
+      </c>
+      <c r="C63" s="23" t="str">
+        <f>C53</f>
+        <v xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </v>
+      </c>
+      <c r="D63" s="26">
+        <f>D58+D59</f>
         <v>109.78</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B57" s="15">
+      <c r="E63" s="27"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B66" s="10"/>
+      <c r="C66" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="30"/>
+      <c r="E66" s="31"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B67" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C67" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E67" s="32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B68" s="15">
+        <v>1</v>
+      </c>
+      <c r="C68" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" s="17">
+        <v>1063.9100000000001</v>
+      </c>
+      <c r="E68" s="32"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B69" s="15">
+        <v>2</v>
+      </c>
+      <c r="C69" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D69" s="17">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="E69" s="32"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B70" s="15">
+        <v>3</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D70" s="17">
+        <v>1063.9100000000001</v>
+      </c>
+      <c r="E70" s="32"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B71" s="15">
         <v>4</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C71" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D57" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="25"/>
-      <c r="B58" s="26">
+      <c r="D71" s="17">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="E71" s="32"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B72" s="15">
         <v>5</v>
       </c>
-      <c r="C58" s="23" t="str">
-        <f>C49</f>
-        <v xml:space="preserve">Окраска поверхности стен с предварительной огрунтовкой в 2 слоя </v>
-      </c>
-      <c r="D58" s="27">
-        <f>D54+D55</f>
-        <v>109.78</v>
-      </c>
-      <c r="E58" s="28"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B61" s="10"/>
-      <c r="C61" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D61" s="31"/>
-      <c r="E61" s="32"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B62" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="E62" s="33" t="s">
+      <c r="C72" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D72" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="32"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B73" s="15">
+        <v>6</v>
+      </c>
+      <c r="C73" s="23" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B63" s="15">
-        <v>1</v>
-      </c>
-      <c r="C63" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D63" s="17">
-        <v>1063.9100000000001</v>
-      </c>
-      <c r="E63" s="33"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B64" s="15">
-        <v>2</v>
-      </c>
-      <c r="C64" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D64" s="17">
-        <v>4.1500000000000004</v>
-      </c>
-      <c r="E64" s="33"/>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="15">
-        <v>3</v>
-      </c>
-      <c r="C65" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D65" s="17">
-        <f>D63+D64</f>
+      <c r="D73" s="17">
+        <f>D68+D69</f>
         <v>1068.0600000000002</v>
       </c>
-      <c r="E65" s="33"/>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B66" s="15">
-        <v>4</v>
-      </c>
-      <c r="C66" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D66" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="E66" s="33"/>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B67" s="34">
-        <v>5</v>
-      </c>
-      <c r="C67" s="23" t="s">
+      <c r="E73" s="32"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B74" s="33">
+        <v>6.1</v>
+      </c>
+      <c r="C74" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D67" s="17">
-        <f>D63+D64</f>
-        <v>1068.0600000000002</v>
-      </c>
-      <c r="E67" s="33"/>
-    </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B68" s="34">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="C68" s="16" t="s">
+      <c r="D74" s="32"/>
+      <c r="E74" s="32">
+        <f>D73*0.15</f>
+        <v>160.20900000000003</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B75" s="33">
+        <v>6.2</v>
+      </c>
+      <c r="C75" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D68" s="33"/>
-      <c r="E68" s="33">
-        <f>D67*0.15</f>
-        <v>160.20900000000003</v>
-      </c>
-    </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B69" s="34">
-        <v>5.2</v>
-      </c>
-      <c r="C69" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="D69" s="33"/>
-      <c r="E69" s="33">
-        <f>D67*0.3</f>
+      <c r="D75" s="32"/>
+      <c r="E75" s="32">
+        <f>D73*0.3</f>
         <v>320.41800000000006</v>
       </c>
     </row>

</xml_diff>